<commit_message>
Cargar la bajada de cargas provisoria en la planilla de columnas
La columna CARGA deja de estar vacia: se carga la bajada automatica
para que la planilla verifique. Queda marcada como provisoria porque
es un piso. Se agrega el estado AL LIMITE cuando la carga supera el
85 por ciento de la capacidad.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_columnas.xlsx
+++ b/planillas/planilla_columnas.xlsx
@@ -991,7 +991,9 @@
       <c r="C4" s="14" t="n">
         <v>3.22</v>
       </c>
-      <c r="D4" s="15" t="n"/>
+      <c r="D4" s="15" t="n">
+        <v>14.25</v>
+      </c>
       <c r="E4" s="16" t="n">
         <v>20</v>
       </c>
@@ -1020,12 +1022,12 @@
         <v/>
       </c>
       <c r="M4" s="6">
-        <f>IF(D4="","FALTA CARGA",IF(O4&lt;H4,"ARM. INSUFIC.",IF(D4&gt;P4,"NO VERIFICA",IF(Q4&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D4="","FALTA CARGA",IF(O4&lt;H4,"ARM. INSUFIC.",IF(D4&gt;P4,"NO VERIFICA",IF(D4&gt;0.85*P4,"AL LIMITE",IF(Q4&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N4" s="18" t="inlineStr">
         <is>
-          <t>COL 07 del plano. Carga estimada por bajada automatica: 14.3 t (incompleta, ver Memoria).</t>
+          <t>COL 07 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O4" s="19">
@@ -1054,7 +1056,9 @@
       <c r="C5" s="14" t="n">
         <v>3.22</v>
       </c>
-      <c r="D5" s="15" t="n"/>
+      <c r="D5" s="15" t="n">
+        <v>17.23</v>
+      </c>
       <c r="E5" s="16" t="n">
         <v>30</v>
       </c>
@@ -1083,12 +1087,12 @@
         <v/>
       </c>
       <c r="M5" s="6">
-        <f>IF(D5="","FALTA CARGA",IF(O5&lt;H5,"ARM. INSUFIC.",IF(D5&gt;P5,"NO VERIFICA",IF(Q5&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D5="","FALTA CARGA",IF(O5&lt;H5,"ARM. INSUFIC.",IF(D5&gt;P5,"NO VERIFICA",IF(D5&gt;0.85*P5,"AL LIMITE",IF(Q5&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N5" s="18" t="inlineStr">
         <is>
-          <t>COL 06 del plano. Carga estimada por bajada automatica: 17.2 t (incompleta, ver Memoria).</t>
+          <t>COL 06 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O5" s="19">
@@ -1117,7 +1121,9 @@
       <c r="C6" s="14" t="n">
         <v>3.22</v>
       </c>
-      <c r="D6" s="15" t="n"/>
+      <c r="D6" s="15" t="n">
+        <v>18.5</v>
+      </c>
       <c r="E6" s="16" t="n">
         <v>15</v>
       </c>
@@ -1146,12 +1152,12 @@
         <v/>
       </c>
       <c r="M6" s="6">
-        <f>IF(D6="","FALTA CARGA",IF(O6&lt;H6,"ARM. INSUFIC.",IF(D6&gt;P6,"NO VERIFICA",IF(Q6&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D6="","FALTA CARGA",IF(O6&lt;H6,"ARM. INSUFIC.",IF(D6&gt;P6,"NO VERIFICA",IF(D6&gt;0.85*P6,"AL LIMITE",IF(Q6&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N6" s="18" t="inlineStr">
         <is>
-          <t>COL 05 del plano. Carga estimada por bajada automatica: 18.5 t (incompleta, ver Memoria).</t>
+          <t>COL 05 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O6" s="19">
@@ -1180,7 +1186,9 @@
       <c r="C7" s="24" t="n">
         <v>3.22</v>
       </c>
-      <c r="D7" s="25" t="n"/>
+      <c r="D7" s="25" t="n">
+        <v>19.44</v>
+      </c>
       <c r="E7" s="26" t="n">
         <v>15</v>
       </c>
@@ -1209,12 +1217,12 @@
         <v/>
       </c>
       <c r="M7" s="27">
-        <f>IF(D7="","FALTA CARGA",IF(O7&lt;H7,"ARM. INSUFIC.",IF(D7&gt;P7,"NO VERIFICA",IF(Q7&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D7="","FALTA CARGA",IF(O7&lt;H7,"ARM. INSUFIC.",IF(D7&gt;P7,"NO VERIFICA",IF(D7&gt;0.85*P7,"AL LIMITE",IF(Q7&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N7" s="29" t="inlineStr">
         <is>
-          <t>COL 05 del plano. Carga estimada por bajada automatica: 19.4 t (incompleta, ver Memoria).</t>
+          <t>COL 05 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O7" s="30">
@@ -1247,7 +1255,9 @@
       <c r="C8" s="14" t="n">
         <v>3.15</v>
       </c>
-      <c r="D8" s="15" t="n"/>
+      <c r="D8" s="15" t="n">
+        <v>6.38</v>
+      </c>
       <c r="E8" s="16" t="n">
         <v>15</v>
       </c>
@@ -1276,12 +1286,12 @@
         <v/>
       </c>
       <c r="M8" s="6">
-        <f>IF(D8="","FALTA CARGA",IF(O8&lt;H8,"ARM. INSUFIC.",IF(D8&gt;P8,"NO VERIFICA",IF(Q8&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D8="","FALTA CARGA",IF(O8&lt;H8,"ARM. INSUFIC.",IF(D8&gt;P8,"NO VERIFICA",IF(D8&gt;0.85*P8,"AL LIMITE",IF(Q8&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N8" s="18" t="inlineStr">
         <is>
-          <t>COL 02 del plano. Carga estimada por bajada automatica: 6.4 t (incompleta, ver Memoria).</t>
+          <t>COL 02 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O8" s="19">
@@ -1310,7 +1320,9 @@
       <c r="C9" s="14" t="n">
         <v>3.15</v>
       </c>
-      <c r="D9" s="15" t="n"/>
+      <c r="D9" s="15" t="n">
+        <v>36.41</v>
+      </c>
       <c r="E9" s="16" t="n">
         <v>15</v>
       </c>
@@ -1339,12 +1351,12 @@
         <v/>
       </c>
       <c r="M9" s="6">
-        <f>IF(D9="","FALTA CARGA",IF(O9&lt;H9,"ARM. INSUFIC.",IF(D9&gt;P9,"NO VERIFICA",IF(Q9&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D9="","FALTA CARGA",IF(O9&lt;H9,"ARM. INSUFIC.",IF(D9&gt;P9,"NO VERIFICA",IF(D9&gt;0.85*P9,"AL LIMITE",IF(Q9&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N9" s="18" t="inlineStr">
         <is>
-          <t>COL 02 del plano. Carga estimada por bajada automatica: 36.4 t (incompleta, ver Memoria).</t>
+          <t>COL 02 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O9" s="19">
@@ -1373,7 +1385,9 @@
       <c r="C10" s="14" t="n">
         <v>3.15</v>
       </c>
-      <c r="D10" s="15" t="n"/>
+      <c r="D10" s="15" t="n">
+        <v>19.85</v>
+      </c>
       <c r="E10" s="16" t="n">
         <v>30</v>
       </c>
@@ -1402,12 +1416,12 @@
         <v/>
       </c>
       <c r="M10" s="6">
-        <f>IF(D10="","FALTA CARGA",IF(O10&lt;H10,"ARM. INSUFIC.",IF(D10&gt;P10,"NO VERIFICA",IF(Q10&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D10="","FALTA CARGA",IF(O10&lt;H10,"ARM. INSUFIC.",IF(D10&gt;P10,"NO VERIFICA",IF(D10&gt;0.85*P10,"AL LIMITE",IF(Q10&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N10" s="18" t="inlineStr">
         <is>
-          <t>COL 03 del plano. Carga estimada por bajada automatica: 19.8 t (incompleta, ver Memoria).</t>
+          <t>COL 03 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O10" s="19">
@@ -1436,7 +1450,9 @@
       <c r="C11" s="14" t="n">
         <v>3.15</v>
       </c>
-      <c r="D11" s="15" t="n"/>
+      <c r="D11" s="15" t="n">
+        <v>28.77</v>
+      </c>
       <c r="E11" s="16" t="n">
         <v>10</v>
       </c>
@@ -1465,12 +1481,12 @@
         <v/>
       </c>
       <c r="M11" s="6">
-        <f>IF(D11="","FALTA CARGA",IF(O11&lt;H11,"ARM. INSUFIC.",IF(D11&gt;P11,"NO VERIFICA",IF(Q11&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D11="","FALTA CARGA",IF(O11&lt;H11,"ARM. INSUFIC.",IF(D11&gt;P11,"NO VERIFICA",IF(D11&gt;0.85*P11,"AL LIMITE",IF(Q11&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N11" s="18" t="inlineStr">
         <is>
-          <t>COL 01 del plano. Carga estimada por bajada automatica: 28.8 t (incompleta, ver Memoria). ATENCION: seccion 10x10 leida del plano. Recibe VI 01a (17 t): una columna de 10x10 no puede tomar esa carga. Probablemente VI 01a apoye en la medianera y esto no sea columna.</t>
+          <t>COL 01 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5). ATENCION: seccion 10x10 leida del plano. Recibe VI 01a (17 t): una columna de 10x10 no puede tomar esa carga. Probablemente VI 01a apoye en la medianera y esto no sea columna.</t>
         </is>
       </c>
       <c r="O11" s="19">
@@ -1499,7 +1515,9 @@
       <c r="C12" s="14" t="n">
         <v>3.15</v>
       </c>
-      <c r="D12" s="15" t="n"/>
+      <c r="D12" s="15" t="n">
+        <v>20.2</v>
+      </c>
       <c r="E12" s="16" t="n">
         <v>15</v>
       </c>
@@ -1528,12 +1546,12 @@
         <v/>
       </c>
       <c r="M12" s="6">
-        <f>IF(D12="","FALTA CARGA",IF(O12&lt;H12,"ARM. INSUFIC.",IF(D12&gt;P12,"NO VERIFICA",IF(Q12&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D12="","FALTA CARGA",IF(O12&lt;H12,"ARM. INSUFIC.",IF(D12&gt;P12,"NO VERIFICA",IF(D12&gt;0.85*P12,"AL LIMITE",IF(Q12&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N12" s="18" t="inlineStr">
         <is>
-          <t>COL 02 del plano. Carga estimada por bajada automatica: 20.2 t (incompleta, ver Memoria).</t>
+          <t>COL 02 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O12" s="19">
@@ -1562,7 +1580,9 @@
       <c r="C13" s="14" t="n">
         <v>3.15</v>
       </c>
-      <c r="D13" s="15" t="n"/>
+      <c r="D13" s="15" t="n">
+        <v>43.36</v>
+      </c>
       <c r="E13" s="16" t="n">
         <v>20</v>
       </c>
@@ -1591,12 +1611,12 @@
         <v/>
       </c>
       <c r="M13" s="6">
-        <f>IF(D13="","FALTA CARGA",IF(O13&lt;H13,"ARM. INSUFIC.",IF(D13&gt;P13,"NO VERIFICA",IF(Q13&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D13="","FALTA CARGA",IF(O13&lt;H13,"ARM. INSUFIC.",IF(D13&gt;P13,"NO VERIFICA",IF(D13&gt;0.85*P13,"AL LIMITE",IF(Q13&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N13" s="18" t="inlineStr">
         <is>
-          <t>COL 04 del plano. Carga estimada por bajada automatica: 43.4 t (incompleta, ver Memoria).</t>
+          <t>COL 04 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O13" s="19">
@@ -1625,7 +1645,9 @@
       <c r="C14" s="14" t="n">
         <v>3.15</v>
       </c>
-      <c r="D14" s="15" t="n"/>
+      <c r="D14" s="15" t="n">
+        <v>32.38</v>
+      </c>
       <c r="E14" s="16" t="n">
         <v>30</v>
       </c>
@@ -1654,12 +1676,12 @@
         <v/>
       </c>
       <c r="M14" s="6">
-        <f>IF(D14="","FALTA CARGA",IF(O14&lt;H14,"ARM. INSUFIC.",IF(D14&gt;P14,"NO VERIFICA",IF(Q14&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D14="","FALTA CARGA",IF(O14&lt;H14,"ARM. INSUFIC.",IF(D14&gt;P14,"NO VERIFICA",IF(D14&gt;0.85*P14,"AL LIMITE",IF(Q14&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N14" s="18" t="inlineStr">
         <is>
-          <t>COL 03 del plano. Carga estimada por bajada automatica: 32.4 t (incompleta, ver Memoria).</t>
+          <t>COL 03 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O14" s="19">
@@ -1688,7 +1710,9 @@
       <c r="C15" s="14" t="n">
         <v>3.15</v>
       </c>
-      <c r="D15" s="15" t="n"/>
+      <c r="D15" s="15" t="n">
+        <v>42.14</v>
+      </c>
       <c r="E15" s="16" t="n">
         <v>15</v>
       </c>
@@ -1717,12 +1741,12 @@
         <v/>
       </c>
       <c r="M15" s="6">
-        <f>IF(D15="","FALTA CARGA",IF(O15&lt;H15,"ARM. INSUFIC.",IF(D15&gt;P15,"NO VERIFICA",IF(Q15&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D15="","FALTA CARGA",IF(O15&lt;H15,"ARM. INSUFIC.",IF(D15&gt;P15,"NO VERIFICA",IF(D15&gt;0.85*P15,"AL LIMITE",IF(Q15&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N15" s="18" t="inlineStr">
         <is>
-          <t>COL 02 del plano. Carga estimada por bajada automatica: 42.1 t (incompleta, ver Memoria).</t>
+          <t>COL 02 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O15" s="19">
@@ -1751,7 +1775,9 @@
       <c r="C16" s="24" t="n">
         <v>3.15</v>
       </c>
-      <c r="D16" s="25" t="n"/>
+      <c r="D16" s="25" t="n">
+        <v>49.51</v>
+      </c>
       <c r="E16" s="26" t="n">
         <v>15</v>
       </c>
@@ -1780,12 +1806,12 @@
         <v/>
       </c>
       <c r="M16" s="27">
-        <f>IF(D16="","FALTA CARGA",IF(O16&lt;H16,"ARM. INSUFIC.",IF(D16&gt;P16,"NO VERIFICA",IF(Q16&gt;34,"VERIF. ESBELTEZ","VERIFICA"))))</f>
+        <f>IF(D16="","FALTA CARGA",IF(O16&lt;H16,"ARM. INSUFIC.",IF(D16&gt;P16,"NO VERIFICA",IF(D16&gt;0.85*P16,"AL LIMITE",IF(Q16&gt;34,"VERIF. ESBELTEZ","VERIFICA")))))</f>
         <v/>
       </c>
       <c r="N16" s="29" t="inlineStr">
         <is>
-          <t>COL 02 del plano. Carga estimada por bajada automatica: 49.5 t (incompleta, ver Memoria).</t>
+          <t>COL 02 del plano. Carga PROVISORIA por bajada automatica; es un piso, la real es mayor (ver Memoria, punto 5).</t>
         </is>
       </c>
       <c r="O16" s="30">
@@ -1836,6 +1862,9 @@
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
       <formula>"FALTA CARGA"</formula>
     </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="1">
+      <formula>"AL LIMITE"</formula>
+    </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="J4:J16 K4:K16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1853,7 +1882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2043,12 +2072,12 @@
     <row r="24">
       <c r="A24" s="33" t="inlineStr">
         <is>
-          <t>5. CARGAS: FALTA</t>
+          <t>5. CARGAS</t>
         </is>
       </c>
       <c r="B24" s="33" t="inlineStr">
         <is>
-          <t>La columna CARGA (t) esta VACIA y hay que completarla. En la columna auxiliar</t>
+          <t>La columna CARGA (t) viene cargada con una bajada automatica: suma de las</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2085,7 @@
       <c r="A25" s="33" t="inlineStr"/>
       <c r="B25" s="34" t="inlineStr">
         <is>
-          <t>carga estim. se deja una bajada automatica, hecha sumando las reacciones de las</t>
+          <t>reacciones de las vigas que apoyan en cada columna (tomadas de la planilla de</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2093,7 @@
       <c r="A26" s="33" t="inlineStr"/>
       <c r="B26" s="34" t="inlineStr">
         <is>
-          <t>vigas ya calculadas mas el peso propio y lo que baja del nivel superior.</t>
+          <t>vigas), mas el peso propio, mas lo que baja de la columna del nivel superior.</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2101,7 @@
       <c r="A27" s="33" t="inlineStr"/>
       <c r="B27" s="34" t="inlineStr">
         <is>
-          <t>ESA ESTIMACION ES UN PISO, NO EL VALOR REAL: 20 de los 60 extremos de viga no</t>
+          <t>ES UNA CARGA PROVISORIA Y ES UN PISO, NO EL VALOR REAL: 20 de los 60 extremos</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2109,7 @@
       <c r="A28" s="33" t="inlineStr"/>
       <c r="B28" s="34" t="inlineStr">
         <is>
-          <t>pudieron asignarse a ninguna columna (apoyan en otra viga, en un tabique o en la</t>
+          <t>de viga no pudieron asignarse a ninguna columna porque apoyan en otra viga, en</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2117,7 @@
       <c r="A29" s="33" t="inlineStr"/>
       <c r="B29" s="34" t="inlineStr">
         <is>
-          <t>medianera), y esas reacciones no estan sumadas. La carga real es mayor.</t>
+          <t>un tabique o en la medianera, y esas reacciones no estan sumadas.</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2125,7 @@
       <c r="A30" s="33" t="inlineStr"/>
       <c r="B30" s="34" t="inlineStr">
         <is>
-          <t>Ademas son cargas MAYORADAS, coherentes con la planilla de vigas. Si la catedra</t>
+          <t>Para cerrarla hay que indicar, para cada uno de esos 20 extremos, en que apoya.</t>
         </is>
       </c>
     </row>
@@ -2104,39 +2133,39 @@
       <c r="A31" s="33" t="inlineStr"/>
       <c r="B31" s="34" t="inlineStr">
         <is>
-          <t>pide cargas de servicio, dividir por el coeficiente que corresponda.</t>
+          <t>Mientras tanto la columna es editable: al corregir un valor todo recalcula.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="33" t="inlineStr"/>
-      <c r="B32" s="34" t="inlineStr"/>
+      <c r="B32" s="34" t="inlineStr">
+        <is>
+          <t>Ademas son cargas MAYORADAS, coherentes con la planilla de vigas. Si la catedra</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="33" t="inlineStr">
-        <is>
-          <t>6. ESBELTEZ</t>
-        </is>
-      </c>
-      <c r="B33" s="33" t="inlineStr">
-        <is>
-          <t>Todas las columnas son esbeltas: con lado menor de 15 cm y 3,15 m de altura,</t>
+      <c r="A33" s="33" t="inlineStr"/>
+      <c r="B33" s="34" t="inlineStr">
+        <is>
+          <t>pide cargas de servicio, dividir por el coeficiente que corresponda.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="33" t="inlineStr"/>
-      <c r="B34" s="34" t="inlineStr">
-        <is>
-          <t>k lu / r = 70, muy por encima del limite de 34 por debajo del cual se puede</t>
-        </is>
-      </c>
+      <c r="B34" s="34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="33" t="inlineStr"/>
-      <c r="B35" s="34" t="inlineStr">
-        <is>
-          <t>despreciar el pandeo. En la practica el llenado de mamposteria las arriostra, pero</t>
+      <c r="A35" s="33" t="inlineStr">
+        <is>
+          <t>6. ESBELTEZ</t>
+        </is>
+      </c>
+      <c r="B35" s="33" t="inlineStr">
+        <is>
+          <t>Todas las columnas son esbeltas: con lado menor de 15 cm y 3,15 m de altura,</t>
         </is>
       </c>
     </row>
@@ -2144,69 +2173,85 @@
       <c r="A36" s="33" t="inlineStr"/>
       <c r="B36" s="34" t="inlineStr">
         <is>
-          <t>si la catedra lo pide hay que verificar segundo orden. La planilla lo marca.</t>
+          <t>k lu / r = 70, muy por encima del limite de 34 por debajo del cual se puede</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="33" t="inlineStr"/>
-      <c r="B37" s="34" t="inlineStr"/>
+      <c r="B37" s="34" t="inlineStr">
+        <is>
+          <t>despreciar el pandeo. En la practica el llenado de mamposteria las arriostra, pero</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="33" t="inlineStr">
-        <is>
-          <t>7. C4, A REVISAR</t>
-        </is>
-      </c>
-      <c r="B38" s="33" t="inlineStr">
-        <is>
-          <t>C4 figura en el plano como 10x10 y recibe el extremo de VI 01a, con 17 t de</t>
+      <c r="A38" s="33" t="inlineStr"/>
+      <c r="B38" s="34" t="inlineStr">
+        <is>
+          <t>si la catedra lo pide hay que verificar segundo orden. La planilla lo marca.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="33" t="inlineStr"/>
-      <c r="B39" s="34" t="inlineStr">
-        <is>
-          <t>reaccion. Una columna de 10x10 no toma esa carga. VI 01a corre sobre la medianera,</t>
-        </is>
-      </c>
+      <c r="B39" s="34" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="33" t="inlineStr"/>
-      <c r="B40" s="34" t="inlineStr">
-        <is>
-          <t>asi que lo mas probable es que apoye en el muro y ese 10x10 no sea una columna.</t>
+      <c r="A40" s="33" t="inlineStr">
+        <is>
+          <t>7. C4, A REVISAR</t>
+        </is>
+      </c>
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>C4 figura en el plano como 10x10 y recibe el extremo de VI 01a, con 17 t de</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="33" t="inlineStr"/>
-      <c r="B41" s="34" t="inlineStr"/>
+      <c r="B41" s="34" t="inlineStr">
+        <is>
+          <t>reaccion. Una columna de 10x10 no toma esa carga. VI 01a corre sobre la medianera,</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="33" t="inlineStr">
-        <is>
-          <t>LIMITACIONES</t>
-        </is>
-      </c>
-      <c r="B42" s="33" t="inlineStr">
-        <is>
-          <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
+      <c r="A42" s="33" t="inlineStr"/>
+      <c r="B42" s="34" t="inlineStr">
+        <is>
+          <t>asi que lo mas probable es que apoye en el muro y ese 10x10 no sea una columna.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="33" t="inlineStr"/>
-      <c r="B43" s="34" t="inlineStr">
+      <c r="B43" s="34" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="33" t="inlineStr">
+        <is>
+          <t>LIMITACIONES</t>
+        </is>
+      </c>
+      <c r="B44" s="33" t="inlineStr">
+        <is>
+          <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="33" t="inlineStr"/>
+      <c r="B45" s="34" t="inlineStr">
         <is>
           <t>No se verifica flexion compuesta: las columnas de borde reciben momento de las</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="33" t="inlineStr"/>
-      <c r="B44" s="34" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="33" t="inlineStr"/>
+      <c r="B46" s="34" t="inlineStr">
         <is>
           <t>vigas invertidas y trabajan a flexo-compresion, no a compresion simple.</t>
         </is>

</xml_diff>

<commit_message>
VI 01a sin losa y apoyos en tabique confirmados por el proyectista
VI 01a es viga de borde sobre la medianera y no recibe losa: solo
peso propio y mamposteria. Su carga baja de 3042 a 1082 kg/m y la
reaccion de 17,3 a 6,2 t, con lo que la columna COL 01 de 10x10 pasa
a entrar. Se confirman como apoyos en tabique los extremos de
VI 01a, VI 02, VI 07c y VI 11a, que por lo tanto no cargan columna.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_columnas.xlsx
+++ b/planillas/planilla_columnas.xlsx
@@ -1451,7 +1451,7 @@
         <v>3.15</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>28.77</v>
+        <v>17.61</v>
       </c>
       <c r="E11" s="16" t="n">
         <v>10</v>
@@ -1502,7 +1502,7 @@
         <v/>
       </c>
       <c r="R11" s="19" t="n">
-        <v>28.77</v>
+        <v>17.61</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">

</xml_diff>

<commit_message>
Calcular los anchos tributarios reales a partir del reparto de losas
Se reemplaza el supuesto uniforme de 2,00 m por el reparto relevado
en obra: cada viga toma la mitad de la luz de cada losa que apoya en
ella, la luz entera si es voladizo, y la fraccion de Marcus en las
dos losas cruzadas. Diez vigas resultan sin losa.
Con esto VI 02 pasa a no verificar (recibe L02 y L03, B = 2,88 m) y
la columna C9 queda por encima de su capacidad.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_columnas.xlsx
+++ b/planillas/planilla_columnas.xlsx
@@ -992,7 +992,7 @@
         <v>3.22</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>14.25</v>
+        <v>12.71</v>
       </c>
       <c r="E4" s="16" t="n">
         <v>20</v>
@@ -1043,7 +1043,7 @@
         <v/>
       </c>
       <c r="R4" s="19" t="n">
-        <v>14.25</v>
+        <v>12.71</v>
       </c>
     </row>
     <row r="5" ht="17" customHeight="1">
@@ -1057,7 +1057,7 @@
         <v>3.22</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>17.23</v>
+        <v>22.06</v>
       </c>
       <c r="E5" s="16" t="n">
         <v>30</v>
@@ -1108,7 +1108,7 @@
         <v/>
       </c>
       <c r="R5" s="19" t="n">
-        <v>17.23</v>
+        <v>22.06</v>
       </c>
     </row>
     <row r="6" ht="17" customHeight="1">
@@ -1122,7 +1122,7 @@
         <v>3.22</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>18.5</v>
+        <v>15.12</v>
       </c>
       <c r="E6" s="16" t="n">
         <v>15</v>
@@ -1173,7 +1173,7 @@
         <v/>
       </c>
       <c r="R6" s="19" t="n">
-        <v>18.5</v>
+        <v>15.12</v>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1">
@@ -1187,7 +1187,7 @@
         <v>3.22</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>19.44</v>
+        <v>20.05</v>
       </c>
       <c r="E7" s="26" t="n">
         <v>15</v>
@@ -1238,7 +1238,7 @@
         <v/>
       </c>
       <c r="R7" s="30" t="n">
-        <v>19.44</v>
+        <v>20.05</v>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
@@ -1256,7 +1256,7 @@
         <v>3.15</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>6.38</v>
+        <v>2.49</v>
       </c>
       <c r="E8" s="16" t="n">
         <v>15</v>
@@ -1307,7 +1307,7 @@
         <v/>
       </c>
       <c r="R8" s="19" t="n">
-        <v>6.38</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1">
@@ -1321,7 +1321,7 @@
         <v>3.15</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>36.41</v>
+        <v>29.47</v>
       </c>
       <c r="E9" s="16" t="n">
         <v>15</v>
@@ -1372,7 +1372,7 @@
         <v/>
       </c>
       <c r="R9" s="19" t="n">
-        <v>36.41</v>
+        <v>29.47</v>
       </c>
     </row>
     <row r="10" ht="17" customHeight="1">
@@ -1386,7 +1386,7 @@
         <v>3.15</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>19.85</v>
+        <v>10.6</v>
       </c>
       <c r="E10" s="16" t="n">
         <v>30</v>
@@ -1437,7 +1437,7 @@
         <v/>
       </c>
       <c r="R10" s="19" t="n">
-        <v>19.85</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="11" ht="17" customHeight="1">
@@ -1451,7 +1451,7 @@
         <v>3.15</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>17.61</v>
+        <v>10.28</v>
       </c>
       <c r="E11" s="16" t="n">
         <v>10</v>
@@ -1502,7 +1502,7 @@
         <v/>
       </c>
       <c r="R11" s="19" t="n">
-        <v>17.61</v>
+        <v>10.28</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
@@ -1516,7 +1516,7 @@
         <v>3.15</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>20.2</v>
+        <v>15.9</v>
       </c>
       <c r="E12" s="16" t="n">
         <v>15</v>
@@ -1567,7 +1567,7 @@
         <v/>
       </c>
       <c r="R12" s="19" t="n">
-        <v>20.2</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -1581,7 +1581,7 @@
         <v>3.15</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>43.36</v>
+        <v>32.1</v>
       </c>
       <c r="E13" s="16" t="n">
         <v>20</v>
@@ -1632,7 +1632,7 @@
         <v/>
       </c>
       <c r="R13" s="19" t="n">
-        <v>43.36</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -1646,7 +1646,7 @@
         <v>3.15</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>32.38</v>
+        <v>37.23</v>
       </c>
       <c r="E14" s="16" t="n">
         <v>30</v>
@@ -1697,7 +1697,7 @@
         <v/>
       </c>
       <c r="R14" s="19" t="n">
-        <v>32.38</v>
+        <v>37.23</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -1711,7 +1711,7 @@
         <v>3.15</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>42.14</v>
+        <v>43.4</v>
       </c>
       <c r="E15" s="16" t="n">
         <v>15</v>
@@ -1762,7 +1762,7 @@
         <v/>
       </c>
       <c r="R15" s="19" t="n">
-        <v>42.14</v>
+        <v>43.4</v>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
@@ -1776,7 +1776,7 @@
         <v>3.15</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>49.51</v>
+        <v>54.69</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>15</v>
@@ -1827,7 +1827,7 @@
         <v/>
       </c>
       <c r="R16" s="30" t="n">
-        <v>49.51</v>
+        <v>54.69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Computar L02 como alero en la carga de VI 02
L02 es un alero: losa de 9 cm sin piso ni sobrecarga de vivienda,
722 kg/m2 contra 980 del entrepiso. Se computa como 0,59 m de ancho
tributario equivalente en lugar de los 0,80 m reales del voladizo.
VI 02 sigue sin verificar: el peso lo pone L03, no el alero.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_columnas.xlsx
+++ b/planillas/planilla_columnas.xlsx
@@ -1711,7 +1711,7 @@
         <v>3.15</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>43.4</v>
+        <v>42.22</v>
       </c>
       <c r="E15" s="16" t="n">
         <v>15</v>
@@ -1762,7 +1762,7 @@
         <v/>
       </c>
       <c r="R15" s="19" t="n">
-        <v>43.4</v>
+        <v>42.22</v>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">

</xml_diff>

<commit_message>
Corregir las luces de VCH 03a y VCH 03b
VCH 03a pasa de 3,71 a 3,83 m y VCH 03b de 2,13 a 2,15 m, segun
relevamiento. Con esto el borde VI 03c + VCH 03b + VCH 03a suma
9,73 m, practicamente la longitud de VI 02 en el borde opuesto.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_columnas.xlsx
+++ b/planillas/planilla_columnas.xlsx
@@ -1646,7 +1646,7 @@
         <v>3.15</v>
       </c>
       <c r="D14" s="15" t="n">
-        <v>37.23</v>
+        <v>37.27</v>
       </c>
       <c r="E14" s="16" t="n">
         <v>30</v>
@@ -1697,7 +1697,7 @@
         <v/>
       </c>
       <c r="R14" s="19" t="n">
-        <v>37.23</v>
+        <v>37.27</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -1776,7 +1776,7 @@
         <v>3.15</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>54.69</v>
+        <v>54.89</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>15</v>
@@ -1827,7 +1827,7 @@
         <v/>
       </c>
       <c r="R16" s="30" t="n">
-        <v>54.69</v>
+        <v>54.89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>